<commit_message>
Actualiza coordenadas y fotos
</commit_message>
<xml_diff>
--- a/plantilla_complejos_instalaciones.xlsx
+++ b/plantilla_complejos_instalaciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ernest.andreu\Desktop\Mapa interactivo\hotel-gis-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6581FC2-9A6E-4A3E-86A6-D6F4E943A469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AEF0C48-8417-4337-9731-A63A675CF2A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Complejos" sheetId="1" r:id="rId1"/>
@@ -3470,10 +3470,10 @@
         <v>33</v>
       </c>
       <c r="J38" s="4">
-        <v>28</v>
+        <v>28.009219999999999</v>
       </c>
       <c r="K38" s="4">
-        <v>-16.649999999999999</v>
+        <v>-16.652560000000001</v>
       </c>
       <c r="L38" s="2">
         <v>282</v>

</xml_diff>